<commit_message>
more tweaks, cli updates, bump version
</commit_message>
<xml_diff>
--- a/soak/soak-data/examplethemes.xlsx
+++ b/soak/soak-data/examplethemes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benwhalley/dev/soaking/soak/soak-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BC8F11C-7ACE-454A-A440-7BFBA38FB688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7CE446-F694-8244-BEC2-C02AC34BC2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="1320" windowWidth="24660" windowHeight="16500" xr2:uid="{7C8B6C6B-D9D0-1F4A-AA87-7A329A831E0D}"/>
   </bookViews>
@@ -36,28 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>maintaining hope and positive identity amid chronic illness uncertainty</t>
-  </si>
-  <si>
-    <t>experiencing profound gratitude and transformation after recovery</t>
-  </si>
-  <si>
-    <t>managing physical limits and embracing lifestyle changes for sustainable recovery</t>
-  </si>
-  <si>
-    <t>using brain retraining as a hopeful, empowering recovery strategy</t>
-  </si>
-  <si>
-    <t>coping with social isolation and misunderstanding by others</t>
-  </si>
-  <si>
-    <t>developing new spiritual meaning and accepting support during illness</t>
-  </si>
-  <si>
-    <t>regulating energy and emotional wellbeing amid chronic illness</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>A</t>
   </si>
@@ -65,35 +44,62 @@
     <t>B</t>
   </si>
   <si>
-    <t>Enduring existential loss, fear, and identity disruption through illness</t>
-  </si>
-  <si>
-    <t>Reclaiming agency and responsibility as a foundation for recovery</t>
-  </si>
-  <si>
-    <t>Transforming emotional turbulence through mindset shifts and self-compassion</t>
-  </si>
-  <si>
-    <t>Regulating the nervous system and processing emotion as therapeutic core</t>
-  </si>
-  <si>
-    <t>Adapting and individualizing recovery through experimentation and flexibility</t>
-  </si>
-  <si>
-    <t>The transformational power of community, hope, and peer stories</t>
-  </si>
-  <si>
-    <t>Illness and recovery as catalysts for identity and value transformation</t>
-  </si>
-  <si>
-    <t>Sustaining recovery through pacing, ongoing growth, and self-stewardship</t>
+    <t>Feeling seen without judgement -- relief and safety in expressing distress without fear of evaluation or burdening others</t>
+  </si>
+  <si>
+    <t>Restoring a sense of agency -- organising thoughts and actions helps counter feelings of helplessness during stress</t>
+  </si>
+  <si>
+    <t>Emotional containment and calm -- interaction dampens anxiety and prevents emotional escalation</t>
+  </si>
+  <si>
+    <t>Private space for sense-making -- the tool is used to reflect, rehearse thoughts, and clarify feelings</t>
+  </si>
+  <si>
+    <t>Managing workload and time pressure -- the tool is framed as a practical aid for planning, prioritising, and coping with academic demands</t>
+  </si>
+  <si>
+    <t>Reducing social costs of support-seeking -- avoids stigma, awkwardness, or obligation associated with asking people for help</t>
+  </si>
+  <si>
+    <t>Normalising stress as situational -- distress is interpreted as a reasonable response to university pressures rather than personal weakness</t>
+  </si>
+  <si>
+    <t>Supplementing rather than replacing human support -- the tool is positioned as a stopgap or complement when other support is unavailable</t>
+  </si>
+  <si>
+    <t>Momentary relief -- short interactions take the edge off stress without producing lasting change</t>
+  </si>
+  <si>
+    <t>Prompted reflection -- questions nudge users to articulate thoughts they had been avoiding</t>
+  </si>
+  <si>
+    <t>Low-effort coping -- support is accessed quickly with minimal emotional or cognitive cost</t>
+  </si>
+  <si>
+    <t>Emotional offloading -- distress is eased by putting worries into words rather than solving them</t>
+  </si>
+  <si>
+    <t>Limited personalisation -- responses feel broadly relevant but not deeply tailored</t>
+  </si>
+  <si>
+    <t>Trust through predictability -- consistent tone and structure make the interaction feel safe</t>
+  </si>
+  <si>
+    <t>Bounded usefulness -- benefits are clearest for mild or moderate stress, not crisis situations</t>
+  </si>
+  <si>
+    <t>Background companion -- the tool sits alongside daily life rather than becoming a focal support</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -106,6 +112,18 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="-webkit-standard"/>
     </font>
   </fonts>
   <fills count="2">
@@ -128,9 +146,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,76 +485,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7EBC59-6B8D-794E-A42D-83F9EF3F97F9}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="1" t="s">
+    <row r="6" spans="1:3" ht="18">
+      <c r="B6" s="1"/>
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1" t="s">
+    <row r="7" spans="1:3" ht="18">
+      <c r="B7" s="1"/>
+      <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
+    <row r="8" spans="1:3" ht="18">
+      <c r="B8" s="1"/>
+      <c r="C8" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="18">
+      <c r="B9" s="1"/>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>